<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-24 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7852,7 +7852,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
@@ -7897,7 +7897,7 @@
     <t>BIOLOGIA,ENGENHARIA AMBIENTAL,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>BIOLOGIA,RESÍDUOS SÓLIDOS,ENGENHARIA AMBIENTAL</t>
+    <t>RESÍDUOS SÓLIDOS,BIOLOGIA,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
     <t>MEDICINA LEGAL,SAÚDE</t>
@@ -7921,7 +7921,7 @@
     <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
-    <t>ENGENHARIA QUÍMICA,ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE CONTÁBIL</t>
@@ -7930,13 +7930,13 @@
     <t>RECURSOS HÍDRICOS,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,BIOLOGIA</t>
-  </si>
-  <si>
     <t>ASSISTÊNCIA SOCIAL,EDIFICAÇÕES</t>
   </si>
   <si>
-    <t>PSICOLOGIA,ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS,SAÚDE,ORÇAMENTO,ASSISTÊNCIA SOCIAL,URBANISMO,SAÚDE MENTAL,ECONOMIA,MOBILIDADE E TRANSPORTE</t>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>MOBILIDADE E TRANSPORTE,SAÚDE,ECONOMICIDADE CONTÁBIL,ECONOMIA,ASSISTÊNCIA SOCIAL,ORÇAMENTO,SAÚDE MENTAL,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,URBANISMO</t>
   </si>
 </sst>
 </file>
@@ -15763,7 +15763,7 @@
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B214" t="s">
         <v>253</v>
@@ -15784,7 +15784,7 @@
         <v>1618</v>
       </c>
       <c r="I214" t="s">
-        <v>1697</v>
+        <v>1643</v>
       </c>
       <c r="J214" t="s">
         <v>1971</v>
@@ -31615,7 +31615,7 @@
         <v>2440</v>
       </c>
       <c r="L664" t="s">
-        <v>2638</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="665" spans="1:12">
@@ -31685,7 +31685,7 @@
         <v>2554</v>
       </c>
       <c r="L666" t="s">
-        <v>2615</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="667" spans="1:12">
@@ -31755,7 +31755,7 @@
         <v>2449</v>
       </c>
       <c r="L668" t="s">
-        <v>2615</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="669" spans="1:12">
@@ -31790,7 +31790,7 @@
         <v>2467</v>
       </c>
       <c r="L669" t="s">
-        <v>2615</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="670" spans="1:12">
@@ -31825,7 +31825,7 @@
         <v>2503</v>
       </c>
       <c r="L670" t="s">
-        <v>2615</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="671" spans="1:12">
@@ -31895,7 +31895,7 @@
         <v>2443</v>
       </c>
       <c r="L672" t="s">
-        <v>2615</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="673" spans="1:12">
@@ -32041,7 +32041,7 @@
         <v>2555</v>
       </c>
       <c r="L676" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="677" spans="1:12">
@@ -32143,7 +32143,7 @@
         <v>2556</v>
       </c>
       <c r="L679" t="s">
-        <v>2617</v>
+        <v>2639</v>
       </c>
     </row>
     <row r="680" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-25 02:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -29126,7 +29126,7 @@
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B597" t="s">
         <v>633</v>
@@ -29150,7 +29150,7 @@
         <v>1612</v>
       </c>
       <c r="I597" t="s">
-        <v>1684</v>
+        <v>1626</v>
       </c>
       <c r="J597" t="s">
         <v>2330</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-25 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -5278,13 +5278,13 @@
     <t>IZABEL REGINA BENITE AGUIAR DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
   </si>
   <si>
+    <t>REINALDO DE SOUZA MACHADO,RONALDO PEIXOTO VELLOSO</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,THIAGO JOSÉ DUPRAT FORTES,VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
     <t>VÍTOR MENDONÇA CELANE PINHEIRO</t>
-  </si>
-  <si>
-    <t>REINALDO DE SOUZA MACHADO,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,THIAGO JOSÉ DUPRAT FORTES,VANESSA TRINDADE CAMPOS DA SILVA</t>
   </si>
   <si>
     <t>JULIANA MARTINS BAHIENSE,RODRIGO VALENTE SERRA</t>
@@ -11464,7 +11464,7 @@
         <v>1612</v>
       </c>
       <c r="I91" t="s">
-        <v>1639</v>
+        <v>1644</v>
       </c>
       <c r="J91" t="s">
         <v>1848</v>
@@ -27002,7 +27002,7 @@
         <v>1612</v>
       </c>
       <c r="I534" t="s">
-        <v>1639</v>
+        <v>1644</v>
       </c>
       <c r="J534" t="s">
         <v>2284</v>
@@ -29916,7 +29916,7 @@
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B617" t="s">
         <v>653</v>
@@ -29937,7 +29937,7 @@
         <v>1612</v>
       </c>
       <c r="I617" t="s">
-        <v>1754</v>
+        <v>1639</v>
       </c>
       <c r="J617" t="s">
         <v>2364</v>
@@ -30045,7 +30045,7 @@
         <v>1631</v>
       </c>
       <c r="I620" t="s">
-        <v>1755</v>
+        <v>1754</v>
       </c>
       <c r="J620" t="s">
         <v>2367</v>
@@ -30185,7 +30185,7 @@
         <v>1612</v>
       </c>
       <c r="I624" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="J624" t="s">
         <v>2371</v>
@@ -30220,7 +30220,7 @@
         <v>1612</v>
       </c>
       <c r="I625" t="s">
-        <v>1756</v>
+        <v>1755</v>
       </c>
       <c r="J625" t="s">
         <v>2371</v>
@@ -30255,7 +30255,7 @@
         <v>1612</v>
       </c>
       <c r="I626" t="s">
-        <v>1754</v>
+        <v>1756</v>
       </c>
       <c r="J626" t="s">
         <v>2372</v>
@@ -30573,7 +30573,7 @@
         <v>1612</v>
       </c>
       <c r="I635" t="s">
-        <v>1754</v>
+        <v>1756</v>
       </c>
       <c r="J635" t="s">
         <v>2381</v>
@@ -31177,7 +31177,7 @@
         <v>1633</v>
       </c>
       <c r="I652" t="s">
-        <v>1754</v>
+        <v>1756</v>
       </c>
       <c r="J652" t="s">
         <v>1792</v>
@@ -31959,7 +31959,7 @@
         <v>1631</v>
       </c>
       <c r="I674" t="s">
-        <v>1754</v>
+        <v>1756</v>
       </c>
       <c r="J674" t="s">
         <v>2415</v>
@@ -32035,7 +32035,7 @@
         <v>1624</v>
       </c>
       <c r="I676" t="s">
-        <v>1754</v>
+        <v>1756</v>
       </c>
       <c r="J676" t="s">
         <v>2417</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-26 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7834,7 +7834,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
@@ -7888,7 +7888,7 @@
     <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
@@ -7909,21 +7909,21 @@
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
+    <t>PATRIMÔNIO HISTÓRICO E CULTURAL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
     <t>RECURSOS HÍDRICOS,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>ASSISTÊNCIA SOCIAL,EDIFICAÇÕES</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE OBRAS,AVALIAÇÃO DE IMÓVEIS</t>
+    <t>EDIFICAÇÕES,ASSISTÊNCIA SOCIAL</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
   </si>
   <si>
-    <t>URBANISMO,BIOLOGIA</t>
-  </si>
-  <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
   </si>
   <si>
@@ -7933,7 +7933,7 @@
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,SAÚDE MENTAL,MOBILIDADE E TRANSPORTE,PSICOLOGIA,ORÇAMENTO,ECONOMICIDADE CONTÁBIL,URBANISMO,SAÚDE,ECONOMIA</t>
+    <t>AVALIAÇÃO DE IMÓVEIS,MOBILIDADE E TRANSPORTE,ORÇAMENTO,SAÚDE MENTAL,ECONOMIA,ECONOMICIDADE CONTÁBIL,URBANISMO,ASSISTÊNCIA SOCIAL,SAÚDE,PSICOLOGIA</t>
   </si>
 </sst>
 </file>
@@ -30591,7 +30591,7 @@
         <v>2544</v>
       </c>
       <c r="L635" t="s">
-        <v>2613</v>
+        <v>2631</v>
       </c>
     </row>
     <row r="636" spans="1:12">
@@ -30772,7 +30772,7 @@
         <v>2436</v>
       </c>
       <c r="L640" t="s">
-        <v>2631</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="641" spans="1:12">
@@ -31195,7 +31195,7 @@
         <v>2547</v>
       </c>
       <c r="L652" t="s">
-        <v>2632</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="653" spans="1:12">
@@ -31230,7 +31230,7 @@
         <v>2452</v>
       </c>
       <c r="L653" t="s">
-        <v>2609</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="654" spans="1:12">
@@ -31338,7 +31338,7 @@
         <v>2467</v>
       </c>
       <c r="L656" t="s">
-        <v>2633</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="657" spans="1:12">
@@ -31411,7 +31411,7 @@
         <v>2430</v>
       </c>
       <c r="L658" t="s">
-        <v>2634</v>
+        <v>2635</v>
       </c>
     </row>
     <row r="659" spans="1:12">
@@ -31449,7 +31449,7 @@
         <v>2441</v>
       </c>
       <c r="L659" t="s">
-        <v>2635</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="660" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-27 12:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4975,129 +4975,129 @@
     <t>LILIAN ALVES DE ARAUJO</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
+    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>REGINA SILBERSTEIN RACHEVSKY</t>
+  </si>
+  <si>
+    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
+  </si>
+  <si>
+    <t>ROSEMARY PROVENZANO THAMI</t>
+  </si>
+  <si>
+    <t>MANOELA DE MORAES SILVA</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,PATRICIA PASSARO DA SILVA TOLEDO</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER,SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>LUZIA LAMOSA ARANTES</t>
+  </si>
+  <si>
+    <t>RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>VICTOR AUGUSTO LOURO BERBARA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING,JORGE LUIS DANTAS BATISTA</t>
+  </si>
+  <si>
+    <t>PEDRO MARCELO ROCHA GOMES</t>
+  </si>
+  <si>
+    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE</t>
+  </si>
+  <si>
+    <t>CASSIA CRISTINA DA SILVA</t>
+  </si>
+  <si>
+    <t>ITAMAR COSTA KALIL</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
+  </si>
+  <si>
+    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO,ROMULO LUCIANO INOCENCIO</t>
+  </si>
+  <si>
+    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>EDUARDO COUTO SOLEDADE</t>
+  </si>
+  <si>
+    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
+  </si>
+  <si>
+    <t>DAGER SALLES AMARAL</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO</t>
+  </si>
+  <si>
+    <t>CARLOS FELIPE DA GRAÇA SILVA</t>
+  </si>
+  <si>
     <t>JORGE LUIS DANTAS BATISTA</t>
   </si>
   <si>
-    <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>REGINA SILBERSTEIN RACHEVSKY</t>
-  </si>
-  <si>
-    <t>ANDRÉA ALVARENGA D´ALMEIDA MORAIS,CELSO SOARES BELFORT GARCIA</t>
-  </si>
-  <si>
-    <t>ROSEMARY PROVENZANO THAMI</t>
-  </si>
-  <si>
-    <t>MANOELA DE MORAES SILVA</t>
-  </si>
-  <si>
-    <t>LILIAN ALVES DE ARAUJO,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,PATRICIA PASSARO DA SILVA TOLEDO</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER,SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>LUZIA LAMOSA ARANTES</t>
-  </si>
-  <si>
-    <t>RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>VICTOR AUGUSTO LOURO BERBARA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,THIAGO JOSÉ DUPRAT FORTES, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,DANIEL FONTANA OBERLING,JORGE LUIS DANTAS BATISTA</t>
-  </si>
-  <si>
-    <t>PEDRO MARCELO ROCHA GOMES</t>
-  </si>
-  <si>
-    <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>CLAUDIA DA SILVA LUNARDI,RENATA PASCOAL FREIRE</t>
-  </si>
-  <si>
-    <t>CASSIA CRISTINA DA SILVA</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
-  </si>
-  <si>
-    <t>ITAMAR COSTA KALIL</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,MAYRA LIMA VERISSIMO RAMOS MUNIVE</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER</t>
-  </si>
-  <si>
-    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO,ROMULO LUCIANO INOCENCIO</t>
-  </si>
-  <si>
-    <t>ALEXANDER MAGNO BORGES GOMES DA SILVA</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA,MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>EDUARDO COUTO SOLEDADE</t>
-  </si>
-  <si>
-    <t>ERIKA SILVEIRA PAES BARRETO ALVES</t>
-  </si>
-  <si>
-    <t>DAGER SALLES AMARAL</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO</t>
-  </si>
-  <si>
-    <t>CARLOS FELIPE DA GRAÇA SILVA</t>
-  </si>
-  <si>
     <t>DANIEL FONTANA OBERLING</t>
   </si>
   <si>
@@ -5176,33 +5176,33 @@
     <t>HELENA FERREIRA DE LIMA</t>
   </si>
   <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>SERGIO PEDRO LOPES</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>ROMULO LUCIANO INOCENCIO</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT</t>
+  </si>
+  <si>
+    <t>MARCELO KOLBLINGER DE GODOY</t>
+  </si>
+  <si>
+    <t>SEZISNANDO JOSE PRIMO PAES</t>
+  </si>
+  <si>
     <t>FERNANDA TEIXEIRA ROSALBA</t>
   </si>
   <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>SERGIO PEDRO LOPES</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>ROMULO LUCIANO INOCENCIO</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT</t>
-  </si>
-  <si>
-    <t>MARCELO KOLBLINGER DE GODOY</t>
-  </si>
-  <si>
-    <t>SEZISNANDO JOSE PRIMO PAES</t>
-  </si>
-  <si>
     <t>MOEMA BELLONI SCHMIDT</t>
   </si>
   <si>
@@ -7822,7 +7822,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
@@ -7855,7 +7855,7 @@
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>ECONOMICIDADE OBRAS,RECURSOS HÍDRICOS</t>
@@ -7894,19 +7894,19 @@
     <t>RECURSOS HÍDRICOS,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>ASSISTÊNCIA SOCIAL,EDIFICAÇÕES</t>
+    <t>EDIFICAÇÕES,ASSISTÊNCIA SOCIAL</t>
   </si>
   <si>
     <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
+    <t>URBANISMO,BIOLOGIA</t>
   </si>
   <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>SAÚDE MENTAL,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS,MOBILIDADE E TRANSPORTE,URBANISMO,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,SAÚDE,ASSISTÊNCIA SOCIAL,ECONOMIA</t>
+    <t>URBANISMO,ECONOMICIDADE CONTÁBIL,ORÇAMENTO,SAÚDE MENTAL,PSICOLOGIA,ECONOMIA,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS,ASSISTÊNCIA SOCIAL,SAÚDE</t>
   </si>
 </sst>
 </file>
@@ -10165,7 +10165,7 @@
     </row>
     <row r="55" spans="1:12">
       <c r="A55" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B55" t="s">
         <v>94</v>
@@ -10361,7 +10361,7 @@
         <v>1612</v>
       </c>
       <c r="I60" t="s">
-        <v>1638</v>
+        <v>1653</v>
       </c>
       <c r="J60" t="s">
         <v>1818</v>
@@ -12636,7 +12636,7 @@
         <v>1612</v>
       </c>
       <c r="I125" t="s">
-        <v>1674</v>
+        <v>1653</v>
       </c>
       <c r="J125" t="s">
         <v>1882</v>
@@ -12671,7 +12671,7 @@
         <v>1612</v>
       </c>
       <c r="I126" t="s">
-        <v>1675</v>
+        <v>1674</v>
       </c>
       <c r="J126" t="s">
         <v>1883</v>
@@ -12741,7 +12741,7 @@
         <v>1612</v>
       </c>
       <c r="I128" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J128" t="s">
         <v>1885</v>
@@ -12951,7 +12951,7 @@
         <v>1612</v>
       </c>
       <c r="I134" t="s">
-        <v>1677</v>
+        <v>1676</v>
       </c>
       <c r="J134" t="s">
         <v>1891</v>
@@ -13021,7 +13021,7 @@
         <v>1612</v>
       </c>
       <c r="I136" t="s">
-        <v>1678</v>
+        <v>1677</v>
       </c>
       <c r="J136" t="s">
         <v>1893</v>
@@ -13091,7 +13091,7 @@
         <v>1612</v>
       </c>
       <c r="I138" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
       <c r="J138" t="s">
         <v>1895</v>
@@ -13126,7 +13126,7 @@
         <v>1612</v>
       </c>
       <c r="I139" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="J139" t="s">
         <v>1896</v>
@@ -13161,7 +13161,7 @@
         <v>1612</v>
       </c>
       <c r="I140" t="s">
-        <v>1681</v>
+        <v>1680</v>
       </c>
       <c r="J140" t="s">
         <v>1897</v>
@@ -13231,7 +13231,7 @@
         <v>1612</v>
       </c>
       <c r="I142" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="J142" t="s">
         <v>1899</v>
@@ -13406,7 +13406,7 @@
         <v>1612</v>
       </c>
       <c r="I147" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J147" t="s">
         <v>1904</v>
@@ -13546,7 +13546,7 @@
         <v>1612</v>
       </c>
       <c r="I151" t="s">
-        <v>1684</v>
+        <v>1683</v>
       </c>
       <c r="J151" t="s">
         <v>1908</v>
@@ -13654,7 +13654,7 @@
         <v>1612</v>
       </c>
       <c r="I154" t="s">
-        <v>1685</v>
+        <v>1684</v>
       </c>
       <c r="J154" t="s">
         <v>1911</v>
@@ -13794,7 +13794,7 @@
         <v>1612</v>
       </c>
       <c r="I158" t="s">
-        <v>1686</v>
+        <v>1685</v>
       </c>
       <c r="J158" t="s">
         <v>1915</v>
@@ -13829,7 +13829,7 @@
         <v>1612</v>
       </c>
       <c r="I159" t="s">
-        <v>1687</v>
+        <v>1686</v>
       </c>
       <c r="J159" t="s">
         <v>1916</v>
@@ -13899,7 +13899,7 @@
         <v>1612</v>
       </c>
       <c r="I161" t="s">
-        <v>1688</v>
+        <v>1687</v>
       </c>
       <c r="J161" t="s">
         <v>1918</v>
@@ -13969,7 +13969,7 @@
         <v>1612</v>
       </c>
       <c r="I163" t="s">
-        <v>1689</v>
+        <v>1688</v>
       </c>
       <c r="J163" t="s">
         <v>1920</v>
@@ -14109,7 +14109,7 @@
         <v>1612</v>
       </c>
       <c r="I167" t="s">
-        <v>1690</v>
+        <v>1689</v>
       </c>
       <c r="J167" t="s">
         <v>1924</v>
@@ -14144,7 +14144,7 @@
         <v>1612</v>
       </c>
       <c r="I168" t="s">
-        <v>1691</v>
+        <v>1690</v>
       </c>
       <c r="J168" t="s">
         <v>1925</v>
@@ -14284,7 +14284,7 @@
         <v>1612</v>
       </c>
       <c r="I172" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="J172" t="s">
         <v>1929</v>
@@ -14354,7 +14354,7 @@
         <v>1612</v>
       </c>
       <c r="I174" t="s">
-        <v>1692</v>
+        <v>1691</v>
       </c>
       <c r="J174" t="s">
         <v>1931</v>
@@ -14389,7 +14389,7 @@
         <v>1612</v>
       </c>
       <c r="I175" t="s">
-        <v>1693</v>
+        <v>1692</v>
       </c>
       <c r="J175" t="s">
         <v>1932</v>
@@ -14459,7 +14459,7 @@
         <v>1612</v>
       </c>
       <c r="I177" t="s">
-        <v>1678</v>
+        <v>1677</v>
       </c>
       <c r="J177" t="s">
         <v>1934</v>
@@ -14739,7 +14739,7 @@
         <v>1612</v>
       </c>
       <c r="I185" t="s">
-        <v>1653</v>
+        <v>1693</v>
       </c>
       <c r="J185" t="s">
         <v>1941</v>
@@ -14949,7 +14949,7 @@
         <v>1612</v>
       </c>
       <c r="I191" t="s">
-        <v>1688</v>
+        <v>1687</v>
       </c>
       <c r="J191" t="s">
         <v>1947</v>
@@ -15544,7 +15544,7 @@
         <v>1612</v>
       </c>
       <c r="I208" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J208" t="s">
         <v>1963</v>
@@ -15614,7 +15614,7 @@
         <v>1612</v>
       </c>
       <c r="I210" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J210" t="s">
         <v>1965</v>
@@ -16559,7 +16559,7 @@
         <v>1612</v>
       </c>
       <c r="I237" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J237" t="s">
         <v>1992</v>
@@ -16734,7 +16734,7 @@
         <v>1612</v>
       </c>
       <c r="I242" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J242" t="s">
         <v>1997</v>
@@ -17364,7 +17364,7 @@
         <v>1612</v>
       </c>
       <c r="I260" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J260" t="s">
         <v>2015</v>
@@ -17612,7 +17612,7 @@
         <v>1617</v>
       </c>
       <c r="I267" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J267" t="s">
         <v>2022</v>
@@ -18207,7 +18207,7 @@
         <v>1612</v>
       </c>
       <c r="I284" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J284" t="s">
         <v>2039</v>
@@ -18242,7 +18242,7 @@
         <v>1612</v>
       </c>
       <c r="I285" t="s">
-        <v>1685</v>
+        <v>1684</v>
       </c>
       <c r="J285" t="s">
         <v>2040</v>
@@ -18417,7 +18417,7 @@
         <v>1612</v>
       </c>
       <c r="I290" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J290" t="s">
         <v>2045</v>
@@ -18606,7 +18606,7 @@
     </row>
     <row r="296" spans="1:12">
       <c r="A296" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B296" t="s">
         <v>335</v>
@@ -18627,7 +18627,7 @@
         <v>1612</v>
       </c>
       <c r="I296" t="s">
-        <v>1720</v>
+        <v>1638</v>
       </c>
       <c r="J296" t="s">
         <v>2051</v>
@@ -18697,7 +18697,7 @@
         <v>1612</v>
       </c>
       <c r="I298" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J298" t="s">
         <v>2053</v>
@@ -18732,7 +18732,7 @@
         <v>1612</v>
       </c>
       <c r="I299" t="s">
-        <v>1721</v>
+        <v>1720</v>
       </c>
       <c r="J299" t="s">
         <v>2054</v>
@@ -18907,7 +18907,7 @@
         <v>1612</v>
       </c>
       <c r="I304" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J304" t="s">
         <v>2059</v>
@@ -18942,7 +18942,7 @@
         <v>1612</v>
       </c>
       <c r="I305" t="s">
-        <v>1722</v>
+        <v>1721</v>
       </c>
       <c r="J305" t="s">
         <v>2060</v>
@@ -19158,7 +19158,7 @@
         <v>1618</v>
       </c>
       <c r="I311" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J311" t="s">
         <v>2066</v>
@@ -19193,7 +19193,7 @@
         <v>1612</v>
       </c>
       <c r="I312" t="s">
-        <v>1723</v>
+        <v>1722</v>
       </c>
       <c r="J312" t="s">
         <v>2067</v>
@@ -19368,7 +19368,7 @@
         <v>1612</v>
       </c>
       <c r="I317" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J317" t="s">
         <v>2072</v>
@@ -19438,7 +19438,7 @@
         <v>1612</v>
       </c>
       <c r="I319" t="s">
-        <v>1724</v>
+        <v>1723</v>
       </c>
       <c r="J319" t="s">
         <v>2074</v>
@@ -19543,7 +19543,7 @@
         <v>1612</v>
       </c>
       <c r="I322" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="J322" t="s">
         <v>2077</v>
@@ -19578,7 +19578,7 @@
         <v>1612</v>
       </c>
       <c r="I323" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J323" t="s">
         <v>2078</v>
@@ -19613,7 +19613,7 @@
         <v>1612</v>
       </c>
       <c r="I324" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J324" t="s">
         <v>2079</v>
@@ -19648,7 +19648,7 @@
         <v>1612</v>
       </c>
       <c r="I325" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="J325" t="s">
         <v>2080</v>
@@ -19718,7 +19718,7 @@
         <v>1612</v>
       </c>
       <c r="I327" t="s">
-        <v>1728</v>
+        <v>1727</v>
       </c>
       <c r="J327" t="s">
         <v>2082</v>
@@ -19858,7 +19858,7 @@
         <v>1612</v>
       </c>
       <c r="I331" t="s">
-        <v>1720</v>
+        <v>1728</v>
       </c>
       <c r="J331" t="s">
         <v>2086</v>
@@ -20033,7 +20033,7 @@
         <v>1612</v>
       </c>
       <c r="I336" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J336" t="s">
         <v>2091</v>
@@ -20278,7 +20278,7 @@
         <v>1612</v>
       </c>
       <c r="I343" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J343" t="s">
         <v>2098</v>
@@ -20733,7 +20733,7 @@
         <v>1612</v>
       </c>
       <c r="I356" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J356" t="s">
         <v>2111</v>
@@ -21328,7 +21328,7 @@
         <v>1612</v>
       </c>
       <c r="I373" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J373" t="s">
         <v>2128</v>
@@ -21678,7 +21678,7 @@
         <v>1612</v>
       </c>
       <c r="I383" t="s">
-        <v>1727</v>
+        <v>1726</v>
       </c>
       <c r="J383" t="s">
         <v>2138</v>
@@ -21996,7 +21996,7 @@
         <v>1612</v>
       </c>
       <c r="I392" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J392" t="s">
         <v>2147</v>
@@ -22384,7 +22384,7 @@
         <v>1612</v>
       </c>
       <c r="I403" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J403" t="s">
         <v>2158</v>
@@ -22982,7 +22982,7 @@
         <v>1612</v>
       </c>
       <c r="I420" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="J420" t="s">
         <v>2175</v>
@@ -23017,7 +23017,7 @@
         <v>1612</v>
       </c>
       <c r="I421" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J421" t="s">
         <v>2176</v>
@@ -23052,7 +23052,7 @@
         <v>1612</v>
       </c>
       <c r="I422" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J422" t="s">
         <v>2177</v>
@@ -23157,7 +23157,7 @@
         <v>1612</v>
       </c>
       <c r="I425" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J425" t="s">
         <v>2180</v>
@@ -23332,7 +23332,7 @@
         <v>1612</v>
       </c>
       <c r="I430" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J430" t="s">
         <v>2185</v>
@@ -23437,7 +23437,7 @@
         <v>1612</v>
       </c>
       <c r="I433" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J433" t="s">
         <v>2188</v>
@@ -24315,7 +24315,7 @@
         <v>1612</v>
       </c>
       <c r="I458" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J458" t="s">
         <v>2212</v>
@@ -24350,7 +24350,7 @@
         <v>1612</v>
       </c>
       <c r="I459" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J459" t="s">
         <v>2212</v>
@@ -24420,7 +24420,7 @@
         <v>1612</v>
       </c>
       <c r="I461" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J461" t="s">
         <v>2214</v>
@@ -26036,7 +26036,7 @@
         <v>1612</v>
       </c>
       <c r="I507" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J507" t="s">
         <v>2260</v>
@@ -26141,7 +26141,7 @@
         <v>1612</v>
       </c>
       <c r="I510" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J510" t="s">
         <v>2263</v>
@@ -26249,7 +26249,7 @@
         <v>1623</v>
       </c>
       <c r="I513" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
       <c r="J513" t="s">
         <v>2265</v>
@@ -26459,7 +26459,7 @@
         <v>1612</v>
       </c>
       <c r="I519" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J519" t="s">
         <v>2271</v>
@@ -26704,7 +26704,7 @@
         <v>1612</v>
       </c>
       <c r="I526" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J526" t="s">
         <v>2278</v>
@@ -26774,7 +26774,7 @@
         <v>1612</v>
       </c>
       <c r="I528" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J528" t="s">
         <v>2280</v>
@@ -28002,7 +28002,7 @@
         <v>1612</v>
       </c>
       <c r="I563" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J563" t="s">
         <v>2315</v>
@@ -28037,7 +28037,7 @@
         <v>1612</v>
       </c>
       <c r="I564" t="s">
-        <v>1674</v>
+        <v>1653</v>
       </c>
       <c r="J564" t="s">
         <v>2316</v>
@@ -28787,7 +28787,7 @@
         <v>1612</v>
       </c>
       <c r="I585" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J585" t="s">
         <v>2333</v>
@@ -28895,7 +28895,7 @@
         <v>1612</v>
       </c>
       <c r="I588" t="s">
-        <v>1726</v>
+        <v>1725</v>
       </c>
       <c r="J588" t="s">
         <v>2336</v>
@@ -28930,7 +28930,7 @@
         <v>1612</v>
       </c>
       <c r="I589" t="s">
-        <v>1674</v>
+        <v>1653</v>
       </c>
       <c r="J589" t="s">
         <v>2337</v>
@@ -28968,7 +28968,7 @@
         <v>1606</v>
       </c>
       <c r="I590" t="s">
-        <v>1638</v>
+        <v>1653</v>
       </c>
       <c r="J590" t="s">
         <v>2338</v>
@@ -29324,7 +29324,7 @@
         <v>1612</v>
       </c>
       <c r="I600" t="s">
-        <v>1674</v>
+        <v>1653</v>
       </c>
       <c r="J600" t="s">
         <v>2348</v>
@@ -29359,7 +29359,7 @@
         <v>1612</v>
       </c>
       <c r="I601" t="s">
-        <v>1675</v>
+        <v>1674</v>
       </c>
       <c r="J601" t="s">
         <v>2349</v>
@@ -29709,7 +29709,7 @@
         <v>1612</v>
       </c>
       <c r="I611" t="s">
-        <v>1674</v>
+        <v>1653</v>
       </c>
       <c r="J611" t="s">
         <v>2359</v>
@@ -30027,7 +30027,7 @@
         <v>1612</v>
       </c>
       <c r="I620" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J620" t="s">
         <v>2367</v>
@@ -30100,7 +30100,7 @@
         <v>1612</v>
       </c>
       <c r="I622" t="s">
-        <v>1674</v>
+        <v>1653</v>
       </c>
       <c r="J622" t="s">
         <v>2369</v>
@@ -30348,7 +30348,7 @@
         <v>1624</v>
       </c>
       <c r="I629" t="s">
-        <v>1681</v>
+        <v>1680</v>
       </c>
       <c r="J629" t="s">
         <v>2376</v>
@@ -30386,7 +30386,7 @@
         <v>1624</v>
       </c>
       <c r="I630" t="s">
-        <v>1681</v>
+        <v>1680</v>
       </c>
       <c r="J630" t="s">
         <v>2376</v>
@@ -30491,7 +30491,7 @@
         <v>1612</v>
       </c>
       <c r="I633" t="s">
-        <v>1691</v>
+        <v>1690</v>
       </c>
       <c r="J633" t="s">
         <v>2379</v>
@@ -31142,7 +31142,7 @@
         <v>2437</v>
       </c>
       <c r="L651" t="s">
-        <v>2549</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="652" spans="1:12">
@@ -31483,7 +31483,7 @@
         <v>1612</v>
       </c>
       <c r="I661" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J661" t="s">
         <v>2404</v>
@@ -31597,7 +31597,7 @@
         <v>2537</v>
       </c>
       <c r="L664" t="s">
-        <v>2628</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="665" spans="1:12">
@@ -31927,7 +31927,7 @@
         <v>2465</v>
       </c>
       <c r="L673" t="s">
-        <v>2605</v>
+        <v>2570</v>
       </c>
     </row>
     <row r="674" spans="1:12">
@@ -32002,7 +32002,7 @@
     </row>
     <row r="676" spans="1:12">
       <c r="A676" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B676" t="s">
         <v>711</v>
@@ -32023,7 +32023,7 @@
         <v>1612</v>
       </c>
       <c r="I676" t="s">
-        <v>1638</v>
+        <v>1732</v>
       </c>
       <c r="J676" t="s">
         <v>2418</v>
@@ -32037,7 +32037,7 @@
     </row>
     <row r="677" spans="1:12">
       <c r="A677" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B677" t="s">
         <v>712</v>
@@ -32058,7 +32058,7 @@
         <v>1612</v>
       </c>
       <c r="I677" t="s">
-        <v>1638</v>
+        <v>1759</v>
       </c>
       <c r="J677" t="s">
         <v>2419</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-08-31 22:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6791" uniqueCount="2612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6781" uniqueCount="2611">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7826,9 +7826,6 @@
   </si>
   <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE CONTÁBIL</t>
-  </si>
-  <si>
-    <t>PATRIMÔNIO HISTÓRICO E CULTURAL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,VALORAÇÃO DANOS AMBIENTAIS</t>
@@ -8207,7 +8204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L676"/>
+  <dimension ref="A1:L675"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -17464,7 +17461,7 @@
     </row>
     <row r="265" spans="1:12">
       <c r="A265" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B265" t="s">
         <v>306</v>
@@ -17485,7 +17482,7 @@
         <v>1601</v>
       </c>
       <c r="I265" t="s">
-        <v>1649</v>
+        <v>1625</v>
       </c>
       <c r="J265" t="s">
         <v>2004</v>
@@ -29304,13 +29301,13 @@
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B602" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="C602" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="D602" t="s">
         <v>1587</v>
@@ -29325,27 +29322,27 @@
         <v>1601</v>
       </c>
       <c r="I602" t="s">
-        <v>1734</v>
+        <v>1703</v>
       </c>
       <c r="J602" t="s">
-        <v>2333</v>
+        <v>2334</v>
       </c>
       <c r="K602" t="s">
-        <v>2518</v>
+        <v>2473</v>
       </c>
       <c r="L602" t="s">
-        <v>2604</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B603" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="C603" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="D603" t="s">
         <v>1587</v>
@@ -29357,16 +29354,19 @@
         <v>1596</v>
       </c>
       <c r="G603" t="s">
-        <v>1601</v>
+        <v>1602</v>
+      </c>
+      <c r="H603" t="s">
+        <v>1616</v>
       </c>
       <c r="I603" t="s">
-        <v>1703</v>
+        <v>1667</v>
       </c>
       <c r="J603" t="s">
-        <v>2334</v>
+        <v>2335</v>
       </c>
       <c r="K603" t="s">
-        <v>2473</v>
+        <v>2416</v>
       </c>
       <c r="L603" t="s">
         <v>2558</v>
@@ -29389,7 +29389,7 @@
         <v>11</v>
       </c>
       <c r="F604" t="s">
-        <v>1596</v>
+        <v>1598</v>
       </c>
       <c r="G604" t="s">
         <v>1602</v>
@@ -29412,13 +29412,13 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B605" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="C605" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="D605" t="s">
         <v>1587</v>
@@ -29430,33 +29430,30 @@
         <v>1598</v>
       </c>
       <c r="G605" t="s">
-        <v>1602</v>
-      </c>
-      <c r="H605" t="s">
-        <v>1616</v>
+        <v>1601</v>
       </c>
       <c r="I605" t="s">
-        <v>1667</v>
+        <v>1736</v>
       </c>
       <c r="J605" t="s">
-        <v>2335</v>
+        <v>2336</v>
       </c>
       <c r="K605" t="s">
-        <v>2416</v>
+        <v>2413</v>
       </c>
       <c r="L605" t="s">
-        <v>2558</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="606" spans="1:12">
       <c r="A606" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="B606" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="C606" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="D606" t="s">
         <v>1587</v>
@@ -29471,27 +29468,27 @@
         <v>1601</v>
       </c>
       <c r="I606" t="s">
-        <v>1736</v>
+        <v>1676</v>
       </c>
       <c r="J606" t="s">
-        <v>2336</v>
+        <v>2337</v>
       </c>
       <c r="K606" t="s">
         <v>2413</v>
       </c>
       <c r="L606" t="s">
-        <v>2605</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="607" spans="1:12">
       <c r="A607" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B607" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="C607" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="D607" t="s">
         <v>1587</v>
@@ -29500,22 +29497,22 @@
         <v>11</v>
       </c>
       <c r="F607" t="s">
-        <v>1598</v>
+        <v>1596</v>
       </c>
       <c r="G607" t="s">
         <v>1601</v>
       </c>
       <c r="I607" t="s">
-        <v>1676</v>
+        <v>1649</v>
       </c>
       <c r="J607" t="s">
-        <v>2337</v>
+        <v>2338</v>
       </c>
       <c r="K607" t="s">
-        <v>2413</v>
+        <v>2440</v>
       </c>
       <c r="L607" t="s">
-        <v>2563</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -29523,16 +29520,16 @@
         <v>23</v>
       </c>
       <c r="B608" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="C608" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="D608" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="E608">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F608" t="s">
         <v>1596</v>
@@ -29541,27 +29538,27 @@
         <v>1601</v>
       </c>
       <c r="I608" t="s">
-        <v>1649</v>
+        <v>1715</v>
       </c>
       <c r="J608" t="s">
-        <v>2338</v>
+        <v>2339</v>
       </c>
       <c r="K608" t="s">
-        <v>2440</v>
+        <v>2519</v>
       </c>
       <c r="L608" t="s">
-        <v>2526</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="609" spans="1:12">
       <c r="A609" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B609" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="C609" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="D609" t="s">
         <v>1588</v>
@@ -29576,27 +29573,27 @@
         <v>1601</v>
       </c>
       <c r="I609" t="s">
-        <v>1715</v>
+        <v>1735</v>
       </c>
       <c r="J609" t="s">
-        <v>2339</v>
+        <v>2048</v>
       </c>
       <c r="K609" t="s">
-        <v>2519</v>
+        <v>2414</v>
       </c>
       <c r="L609" t="s">
-        <v>2558</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="610" spans="1:12">
       <c r="A610" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B610" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="C610" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="D610" t="s">
         <v>1588</v>
@@ -29611,16 +29608,16 @@
         <v>1601</v>
       </c>
       <c r="I610" t="s">
-        <v>1735</v>
+        <v>1715</v>
       </c>
       <c r="J610" t="s">
-        <v>2048</v>
+        <v>2340</v>
       </c>
       <c r="K610" t="s">
-        <v>2414</v>
+        <v>2422</v>
       </c>
       <c r="L610" t="s">
-        <v>2582</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="611" spans="1:12">
@@ -29628,10 +29625,10 @@
         <v>23</v>
       </c>
       <c r="B611" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C611" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="D611" t="s">
         <v>1588</v>
@@ -29646,13 +29643,13 @@
         <v>1601</v>
       </c>
       <c r="I611" t="s">
-        <v>1715</v>
+        <v>1703</v>
       </c>
       <c r="J611" t="s">
-        <v>2340</v>
+        <v>2341</v>
       </c>
       <c r="K611" t="s">
-        <v>2422</v>
+        <v>2436</v>
       </c>
       <c r="L611" t="s">
         <v>2558</v>
@@ -29663,10 +29660,10 @@
         <v>23</v>
       </c>
       <c r="B612" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C612" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="D612" t="s">
         <v>1588</v>
@@ -29681,27 +29678,27 @@
         <v>1601</v>
       </c>
       <c r="I612" t="s">
-        <v>1703</v>
+        <v>1694</v>
       </c>
       <c r="J612" t="s">
-        <v>2341</v>
+        <v>2342</v>
       </c>
       <c r="K612" t="s">
-        <v>2436</v>
+        <v>2473</v>
       </c>
       <c r="L612" t="s">
-        <v>2558</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="613" spans="1:12">
       <c r="A613" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B613" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="C613" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="D613" t="s">
         <v>1588</v>
@@ -29716,27 +29713,27 @@
         <v>1601</v>
       </c>
       <c r="I613" t="s">
-        <v>1694</v>
+        <v>1735</v>
       </c>
       <c r="J613" t="s">
-        <v>2342</v>
+        <v>2343</v>
       </c>
       <c r="K613" t="s">
-        <v>2473</v>
+        <v>2458</v>
       </c>
       <c r="L613" t="s">
-        <v>2526</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="614" spans="1:12">
       <c r="A614" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B614" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C614" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="D614" t="s">
         <v>1588</v>
@@ -29751,27 +29748,27 @@
         <v>1601</v>
       </c>
       <c r="I614" t="s">
-        <v>1735</v>
+        <v>1703</v>
       </c>
       <c r="J614" t="s">
-        <v>2343</v>
+        <v>2344</v>
       </c>
       <c r="K614" t="s">
-        <v>2458</v>
+        <v>2416</v>
       </c>
       <c r="L614" t="s">
-        <v>2537</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B615" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="C615" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="D615" t="s">
         <v>1588</v>
@@ -29786,27 +29783,27 @@
         <v>1601</v>
       </c>
       <c r="I615" t="s">
-        <v>1703</v>
+        <v>1735</v>
       </c>
       <c r="J615" t="s">
-        <v>2344</v>
+        <v>2345</v>
       </c>
       <c r="K615" t="s">
-        <v>2416</v>
+        <v>2480</v>
       </c>
       <c r="L615" t="s">
-        <v>2558</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B616" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="C616" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="D616" t="s">
         <v>1588</v>
@@ -29821,27 +29818,27 @@
         <v>1601</v>
       </c>
       <c r="I616" t="s">
-        <v>1735</v>
+        <v>1703</v>
       </c>
       <c r="J616" t="s">
-        <v>2345</v>
+        <v>2346</v>
       </c>
       <c r="K616" t="s">
         <v>2480</v>
       </c>
       <c r="L616" t="s">
-        <v>2537</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B617" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C617" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="D617" t="s">
         <v>1588</v>
@@ -29853,19 +29850,22 @@
         <v>1596</v>
       </c>
       <c r="G617" t="s">
-        <v>1601</v>
+        <v>1604</v>
+      </c>
+      <c r="H617" t="s">
+        <v>1617</v>
       </c>
       <c r="I617" t="s">
-        <v>1703</v>
+        <v>1734</v>
       </c>
       <c r="J617" t="s">
-        <v>2346</v>
+        <v>1777</v>
       </c>
       <c r="K617" t="s">
-        <v>2480</v>
+        <v>2520</v>
       </c>
       <c r="L617" t="s">
-        <v>2558</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="618" spans="1:12">
@@ -29873,48 +29873,45 @@
         <v>24</v>
       </c>
       <c r="B618" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="C618" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="D618" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="E618">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F618" t="s">
         <v>1596</v>
       </c>
       <c r="G618" t="s">
-        <v>1604</v>
-      </c>
-      <c r="H618" t="s">
-        <v>1617</v>
+        <v>1601</v>
       </c>
       <c r="I618" t="s">
-        <v>1734</v>
+        <v>1735</v>
       </c>
       <c r="J618" t="s">
-        <v>1777</v>
+        <v>2347</v>
       </c>
       <c r="K618" t="s">
-        <v>2520</v>
+        <v>2429</v>
       </c>
       <c r="L618" t="s">
-        <v>2606</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="619" spans="1:12">
       <c r="A619" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B619" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="C619" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="D619" t="s">
         <v>1589</v>
@@ -29929,16 +29926,16 @@
         <v>1601</v>
       </c>
       <c r="I619" t="s">
-        <v>1735</v>
+        <v>1715</v>
       </c>
       <c r="J619" t="s">
-        <v>2347</v>
+        <v>2348</v>
       </c>
       <c r="K619" t="s">
         <v>2429</v>
       </c>
       <c r="L619" t="s">
-        <v>2560</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29946,34 +29943,37 @@
         <v>23</v>
       </c>
       <c r="B620" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="C620" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="D620" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="E620">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F620" t="s">
         <v>1596</v>
       </c>
       <c r="G620" t="s">
-        <v>1601</v>
+        <v>1603</v>
+      </c>
+      <c r="H620" t="s">
+        <v>1618</v>
       </c>
       <c r="I620" t="s">
-        <v>1715</v>
+        <v>1694</v>
       </c>
       <c r="J620" t="s">
-        <v>2348</v>
+        <v>2349</v>
       </c>
       <c r="K620" t="s">
-        <v>2429</v>
+        <v>2504</v>
       </c>
       <c r="L620" t="s">
-        <v>2558</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="621" spans="1:12">
@@ -29981,10 +29981,10 @@
         <v>23</v>
       </c>
       <c r="B621" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="C621" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="D621" t="s">
         <v>1590</v>
@@ -29996,22 +29996,19 @@
         <v>1596</v>
       </c>
       <c r="G621" t="s">
-        <v>1603</v>
-      </c>
-      <c r="H621" t="s">
-        <v>1618</v>
+        <v>1601</v>
       </c>
       <c r="I621" t="s">
         <v>1694</v>
       </c>
       <c r="J621" t="s">
-        <v>2349</v>
+        <v>2350</v>
       </c>
       <c r="K621" t="s">
-        <v>2504</v>
+        <v>2440</v>
       </c>
       <c r="L621" t="s">
-        <v>2526</v>
+        <v>2606</v>
       </c>
     </row>
     <row r="622" spans="1:12">
@@ -30019,10 +30016,10 @@
         <v>23</v>
       </c>
       <c r="B622" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C622" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="D622" t="s">
         <v>1590</v>
@@ -30037,27 +30034,27 @@
         <v>1601</v>
       </c>
       <c r="I622" t="s">
-        <v>1694</v>
+        <v>1714</v>
       </c>
       <c r="J622" t="s">
-        <v>2350</v>
+        <v>2351</v>
       </c>
       <c r="K622" t="s">
-        <v>2440</v>
+        <v>2443</v>
       </c>
       <c r="L622" t="s">
-        <v>2607</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="623" spans="1:12">
       <c r="A623" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="B623" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="C623" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="D623" t="s">
         <v>1590</v>
@@ -30066,33 +30063,36 @@
         <v>7</v>
       </c>
       <c r="F623" t="s">
-        <v>1596</v>
+        <v>1598</v>
       </c>
       <c r="G623" t="s">
-        <v>1601</v>
+        <v>1602</v>
+      </c>
+      <c r="H623" t="s">
+        <v>1612</v>
       </c>
       <c r="I623" t="s">
-        <v>1714</v>
+        <v>1737</v>
       </c>
       <c r="J623" t="s">
-        <v>2351</v>
+        <v>2352</v>
       </c>
       <c r="K623" t="s">
-        <v>2443</v>
+        <v>2407</v>
       </c>
       <c r="L623" t="s">
-        <v>2582</v>
+        <v>2589</v>
       </c>
     </row>
     <row r="624" spans="1:12">
       <c r="A624" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="B624" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="C624" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="D624" t="s">
         <v>1590</v>
@@ -30107,30 +30107,30 @@
         <v>1602</v>
       </c>
       <c r="H624" t="s">
-        <v>1612</v>
+        <v>1619</v>
       </c>
       <c r="I624" t="s">
-        <v>1737</v>
+        <v>1738</v>
       </c>
       <c r="J624" t="s">
-        <v>2352</v>
+        <v>2353</v>
       </c>
       <c r="K624" t="s">
-        <v>2407</v>
+        <v>2418</v>
       </c>
       <c r="L624" t="s">
-        <v>2589</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="625" spans="1:12">
       <c r="A625" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B625" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C625" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="D625" t="s">
         <v>1590</v>
@@ -30139,25 +30139,22 @@
         <v>7</v>
       </c>
       <c r="F625" t="s">
-        <v>1598</v>
+        <v>1596</v>
       </c>
       <c r="G625" t="s">
-        <v>1602</v>
-      </c>
-      <c r="H625" t="s">
-        <v>1619</v>
+        <v>1601</v>
       </c>
       <c r="I625" t="s">
-        <v>1738</v>
+        <v>1715</v>
       </c>
       <c r="J625" t="s">
-        <v>2353</v>
+        <v>2354</v>
       </c>
       <c r="K625" t="s">
-        <v>2418</v>
+        <v>2483</v>
       </c>
       <c r="L625" t="s">
-        <v>2528</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="626" spans="1:12">
@@ -30165,10 +30162,10 @@
         <v>23</v>
       </c>
       <c r="B626" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C626" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="D626" t="s">
         <v>1590</v>
@@ -30183,16 +30180,16 @@
         <v>1601</v>
       </c>
       <c r="I626" t="s">
-        <v>1715</v>
+        <v>1731</v>
       </c>
       <c r="J626" t="s">
-        <v>2354</v>
+        <v>2355</v>
       </c>
       <c r="K626" t="s">
-        <v>2483</v>
+        <v>2452</v>
       </c>
       <c r="L626" t="s">
-        <v>2558</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="627" spans="1:12">
@@ -30200,10 +30197,10 @@
         <v>23</v>
       </c>
       <c r="B627" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="C627" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="D627" t="s">
         <v>1590</v>
@@ -30218,16 +30215,16 @@
         <v>1601</v>
       </c>
       <c r="I627" t="s">
-        <v>1731</v>
+        <v>1649</v>
       </c>
       <c r="J627" t="s">
-        <v>2355</v>
+        <v>2356</v>
       </c>
       <c r="K627" t="s">
-        <v>2452</v>
+        <v>2448</v>
       </c>
       <c r="L627" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="628" spans="1:12">
@@ -30235,16 +30232,16 @@
         <v>23</v>
       </c>
       <c r="B628" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="C628" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="D628" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="E628">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F628" t="s">
         <v>1596</v>
@@ -30253,16 +30250,16 @@
         <v>1601</v>
       </c>
       <c r="I628" t="s">
-        <v>1649</v>
+        <v>1714</v>
       </c>
       <c r="J628" t="s">
-        <v>2356</v>
+        <v>2357</v>
       </c>
       <c r="K628" t="s">
-        <v>2448</v>
+        <v>2442</v>
       </c>
       <c r="L628" t="s">
-        <v>2526</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30270,10 +30267,10 @@
         <v>23</v>
       </c>
       <c r="B629" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="C629" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="D629" t="s">
         <v>1591</v>
@@ -30288,16 +30285,16 @@
         <v>1601</v>
       </c>
       <c r="I629" t="s">
-        <v>1714</v>
+        <v>1731</v>
       </c>
       <c r="J629" t="s">
-        <v>2357</v>
+        <v>2358</v>
       </c>
       <c r="K629" t="s">
-        <v>2442</v>
+        <v>2435</v>
       </c>
       <c r="L629" t="s">
-        <v>2582</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="630" spans="1:12">
@@ -30305,10 +30302,10 @@
         <v>23</v>
       </c>
       <c r="B630" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C630" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="D630" t="s">
         <v>1591</v>
@@ -30323,27 +30320,27 @@
         <v>1601</v>
       </c>
       <c r="I630" t="s">
-        <v>1731</v>
+        <v>1649</v>
       </c>
       <c r="J630" t="s">
-        <v>2358</v>
+        <v>2359</v>
       </c>
       <c r="K630" t="s">
-        <v>2435</v>
+        <v>2416</v>
       </c>
       <c r="L630" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="631" spans="1:12">
       <c r="A631" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B631" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="C631" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="D631" t="s">
         <v>1591</v>
@@ -30358,27 +30355,27 @@
         <v>1601</v>
       </c>
       <c r="I631" t="s">
-        <v>1649</v>
+        <v>1734</v>
       </c>
       <c r="J631" t="s">
-        <v>2359</v>
+        <v>1762</v>
       </c>
       <c r="K631" t="s">
         <v>2416</v>
       </c>
       <c r="L631" t="s">
-        <v>2526</v>
+        <v>2533</v>
       </c>
     </row>
     <row r="632" spans="1:12">
       <c r="A632" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B632" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="C632" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="D632" t="s">
         <v>1591</v>
@@ -30393,16 +30390,16 @@
         <v>1601</v>
       </c>
       <c r="I632" t="s">
-        <v>1734</v>
+        <v>1714</v>
       </c>
       <c r="J632" t="s">
-        <v>1762</v>
+        <v>2360</v>
       </c>
       <c r="K632" t="s">
-        <v>2416</v>
+        <v>2521</v>
       </c>
       <c r="L632" t="s">
-        <v>2533</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="633" spans="1:12">
@@ -30410,10 +30407,10 @@
         <v>23</v>
       </c>
       <c r="B633" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="C633" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="D633" t="s">
         <v>1591</v>
@@ -30428,16 +30425,16 @@
         <v>1601</v>
       </c>
       <c r="I633" t="s">
-        <v>1714</v>
+        <v>1739</v>
       </c>
       <c r="J633" t="s">
-        <v>2360</v>
+        <v>2361</v>
       </c>
       <c r="K633" t="s">
-        <v>2521</v>
+        <v>2420</v>
       </c>
       <c r="L633" t="s">
-        <v>2582</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -30445,10 +30442,10 @@
         <v>23</v>
       </c>
       <c r="B634" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="C634" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="D634" t="s">
         <v>1591</v>
@@ -30463,10 +30460,10 @@
         <v>1601</v>
       </c>
       <c r="I634" t="s">
-        <v>1739</v>
+        <v>1669</v>
       </c>
       <c r="J634" t="s">
-        <v>2361</v>
+        <v>2362</v>
       </c>
       <c r="K634" t="s">
         <v>2420</v>
@@ -30480,10 +30477,10 @@
         <v>23</v>
       </c>
       <c r="B635" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="C635" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="D635" t="s">
         <v>1591</v>
@@ -30498,16 +30495,16 @@
         <v>1601</v>
       </c>
       <c r="I635" t="s">
-        <v>1669</v>
+        <v>1703</v>
       </c>
       <c r="J635" t="s">
-        <v>2362</v>
+        <v>2363</v>
       </c>
       <c r="K635" t="s">
         <v>2420</v>
       </c>
       <c r="L635" t="s">
-        <v>2526</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="636" spans="1:12">
@@ -30515,10 +30512,10 @@
         <v>23</v>
       </c>
       <c r="B636" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="C636" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="D636" t="s">
         <v>1591</v>
@@ -30536,10 +30533,10 @@
         <v>1703</v>
       </c>
       <c r="J636" t="s">
-        <v>2363</v>
+        <v>2364</v>
       </c>
       <c r="K636" t="s">
-        <v>2420</v>
+        <v>2496</v>
       </c>
       <c r="L636" t="s">
         <v>2558</v>
@@ -30547,13 +30544,13 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B637" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="C637" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="D637" t="s">
         <v>1591</v>
@@ -30568,16 +30565,16 @@
         <v>1601</v>
       </c>
       <c r="I637" t="s">
-        <v>1703</v>
+        <v>1740</v>
       </c>
       <c r="J637" t="s">
-        <v>2364</v>
+        <v>2365</v>
       </c>
       <c r="K637" t="s">
-        <v>2496</v>
+        <v>2515</v>
       </c>
       <c r="L637" t="s">
-        <v>2558</v>
+        <v>2602</v>
       </c>
     </row>
     <row r="638" spans="1:12">
@@ -30585,10 +30582,10 @@
         <v>24</v>
       </c>
       <c r="B638" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="C638" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="D638" t="s">
         <v>1591</v>
@@ -30603,27 +30600,27 @@
         <v>1601</v>
       </c>
       <c r="I638" t="s">
-        <v>1740</v>
+        <v>1735</v>
       </c>
       <c r="J638" t="s">
-        <v>2365</v>
+        <v>2366</v>
       </c>
       <c r="K638" t="s">
-        <v>2515</v>
+        <v>2446</v>
       </c>
       <c r="L638" t="s">
-        <v>2602</v>
+        <v>2607</v>
       </c>
     </row>
     <row r="639" spans="1:12">
       <c r="A639" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B639" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C639" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="D639" t="s">
         <v>1591</v>
@@ -30638,27 +30635,27 @@
         <v>1601</v>
       </c>
       <c r="I639" t="s">
-        <v>1735</v>
+        <v>1649</v>
       </c>
       <c r="J639" t="s">
-        <v>2366</v>
+        <v>2232</v>
       </c>
       <c r="K639" t="s">
-        <v>2446</v>
+        <v>2407</v>
       </c>
       <c r="L639" t="s">
-        <v>2608</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="640" spans="1:12">
       <c r="A640" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="B640" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="C640" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="D640" t="s">
         <v>1591</v>
@@ -30670,30 +30667,33 @@
         <v>1596</v>
       </c>
       <c r="G640" t="s">
-        <v>1601</v>
+        <v>1602</v>
+      </c>
+      <c r="H640" t="s">
+        <v>1615</v>
       </c>
       <c r="I640" t="s">
-        <v>1649</v>
+        <v>1741</v>
       </c>
       <c r="J640" t="s">
-        <v>2232</v>
+        <v>2367</v>
       </c>
       <c r="K640" t="s">
-        <v>2407</v>
+        <v>2489</v>
       </c>
       <c r="L640" t="s">
-        <v>2526</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="641" spans="1:12">
       <c r="A641" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="B641" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="C641" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="D641" t="s">
         <v>1591</v>
@@ -30705,33 +30705,33 @@
         <v>1596</v>
       </c>
       <c r="G641" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="H641" t="s">
-        <v>1615</v>
+        <v>1620</v>
       </c>
       <c r="I641" t="s">
-        <v>1741</v>
+        <v>1714</v>
       </c>
       <c r="J641" t="s">
-        <v>2367</v>
+        <v>2368</v>
       </c>
       <c r="K641" t="s">
-        <v>2489</v>
+        <v>2480</v>
       </c>
       <c r="L641" t="s">
-        <v>2540</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="642" spans="1:12">
       <c r="A642" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B642" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="C642" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="D642" t="s">
         <v>1591</v>
@@ -30740,36 +30740,36 @@
         <v>6</v>
       </c>
       <c r="F642" t="s">
-        <v>1596</v>
+        <v>1598</v>
       </c>
       <c r="G642" t="s">
-        <v>1603</v>
+        <v>1602</v>
       </c>
       <c r="H642" t="s">
-        <v>1620</v>
+        <v>1616</v>
       </c>
       <c r="I642" t="s">
-        <v>1714</v>
+        <v>1690</v>
       </c>
       <c r="J642" t="s">
-        <v>2368</v>
+        <v>2369</v>
       </c>
       <c r="K642" t="s">
-        <v>2480</v>
+        <v>2456</v>
       </c>
       <c r="L642" t="s">
-        <v>2582</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="643" spans="1:12">
       <c r="A643" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B643" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="C643" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="D643" t="s">
         <v>1591</v>
@@ -30778,42 +30778,39 @@
         <v>6</v>
       </c>
       <c r="F643" t="s">
-        <v>1598</v>
+        <v>1596</v>
       </c>
       <c r="G643" t="s">
-        <v>1602</v>
-      </c>
-      <c r="H643" t="s">
-        <v>1616</v>
+        <v>1601</v>
       </c>
       <c r="I643" t="s">
-        <v>1690</v>
+        <v>1735</v>
       </c>
       <c r="J643" t="s">
-        <v>2369</v>
+        <v>2370</v>
       </c>
       <c r="K643" t="s">
-        <v>2456</v>
+        <v>2491</v>
       </c>
       <c r="L643" t="s">
-        <v>2571</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="644" spans="1:12">
       <c r="A644" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B644" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C644" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="D644" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="E644">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F644" t="s">
         <v>1596</v>
@@ -30822,27 +30819,27 @@
         <v>1601</v>
       </c>
       <c r="I644" t="s">
-        <v>1735</v>
+        <v>1714</v>
       </c>
       <c r="J644" t="s">
-        <v>2370</v>
+        <v>2371</v>
       </c>
       <c r="K644" t="s">
-        <v>2491</v>
+        <v>2437</v>
       </c>
       <c r="L644" t="s">
-        <v>2548</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="645" spans="1:12">
       <c r="A645" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B645" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="C645" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="D645" t="s">
         <v>1592</v>
@@ -30851,33 +30848,36 @@
         <v>5</v>
       </c>
       <c r="F645" t="s">
-        <v>1596</v>
+        <v>1598</v>
       </c>
       <c r="G645" t="s">
-        <v>1601</v>
+        <v>1602</v>
+      </c>
+      <c r="H645" t="s">
+        <v>1621</v>
       </c>
       <c r="I645" t="s">
-        <v>1714</v>
+        <v>1742</v>
       </c>
       <c r="J645" t="s">
-        <v>2371</v>
+        <v>2372</v>
       </c>
       <c r="K645" t="s">
-        <v>2437</v>
+        <v>2442</v>
       </c>
       <c r="L645" t="s">
-        <v>2582</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="646" spans="1:12">
       <c r="A646" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="B646" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="C646" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="D646" t="s">
         <v>1592</v>
@@ -30886,36 +30886,33 @@
         <v>5</v>
       </c>
       <c r="F646" t="s">
-        <v>1598</v>
+        <v>1596</v>
       </c>
       <c r="G646" t="s">
-        <v>1602</v>
-      </c>
-      <c r="H646" t="s">
-        <v>1621</v>
+        <v>1601</v>
       </c>
       <c r="I646" t="s">
-        <v>1742</v>
+        <v>1735</v>
       </c>
       <c r="J646" t="s">
-        <v>2372</v>
+        <v>2373</v>
       </c>
       <c r="K646" t="s">
-        <v>2442</v>
+        <v>2478</v>
       </c>
       <c r="L646" t="s">
-        <v>2547</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="647" spans="1:12">
       <c r="A647" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B647" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="C647" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="D647" t="s">
         <v>1592</v>
@@ -30930,16 +30927,16 @@
         <v>1601</v>
       </c>
       <c r="I647" t="s">
-        <v>1735</v>
+        <v>1714</v>
       </c>
       <c r="J647" t="s">
-        <v>2373</v>
+        <v>2374</v>
       </c>
       <c r="K647" t="s">
-        <v>2478</v>
+        <v>2442</v>
       </c>
       <c r="L647" t="s">
-        <v>2609</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="648" spans="1:12">
@@ -30947,16 +30944,16 @@
         <v>23</v>
       </c>
       <c r="B648" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C648" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="D648" t="s">
-        <v>1592</v>
+        <v>1593</v>
       </c>
       <c r="E648">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F648" t="s">
         <v>1596</v>
@@ -30965,16 +30962,16 @@
         <v>1601</v>
       </c>
       <c r="I648" t="s">
-        <v>1714</v>
+        <v>1669</v>
       </c>
       <c r="J648" t="s">
-        <v>2374</v>
+        <v>2375</v>
       </c>
       <c r="K648" t="s">
-        <v>2442</v>
+        <v>2438</v>
       </c>
       <c r="L648" t="s">
-        <v>2582</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="649" spans="1:12">
@@ -30982,10 +30979,10 @@
         <v>23</v>
       </c>
       <c r="B649" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="C649" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="D649" t="s">
         <v>1593</v>
@@ -31003,10 +31000,10 @@
         <v>1669</v>
       </c>
       <c r="J649" t="s">
-        <v>2375</v>
+        <v>2376</v>
       </c>
       <c r="K649" t="s">
-        <v>2438</v>
+        <v>2450</v>
       </c>
       <c r="L649" t="s">
         <v>2526</v>
@@ -31017,10 +31014,10 @@
         <v>23</v>
       </c>
       <c r="B650" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="C650" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="D650" t="s">
         <v>1593</v>
@@ -31035,16 +31032,16 @@
         <v>1601</v>
       </c>
       <c r="I650" t="s">
-        <v>1669</v>
+        <v>1703</v>
       </c>
       <c r="J650" t="s">
-        <v>2376</v>
+        <v>2377</v>
       </c>
       <c r="K650" t="s">
-        <v>2450</v>
+        <v>2473</v>
       </c>
       <c r="L650" t="s">
-        <v>2526</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -31052,10 +31049,10 @@
         <v>23</v>
       </c>
       <c r="B651" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="C651" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="D651" t="s">
         <v>1593</v>
@@ -31070,27 +31067,27 @@
         <v>1601</v>
       </c>
       <c r="I651" t="s">
-        <v>1703</v>
+        <v>1694</v>
       </c>
       <c r="J651" t="s">
-        <v>2377</v>
+        <v>2378</v>
       </c>
       <c r="K651" t="s">
-        <v>2473</v>
+        <v>2483</v>
       </c>
       <c r="L651" t="s">
-        <v>2558</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B652" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="C652" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="D652" t="s">
         <v>1593</v>
@@ -31099,33 +31096,36 @@
         <v>4</v>
       </c>
       <c r="F652" t="s">
-        <v>1596</v>
+        <v>1598</v>
       </c>
       <c r="G652" t="s">
-        <v>1601</v>
+        <v>1602</v>
+      </c>
+      <c r="H652" t="s">
+        <v>1619</v>
       </c>
       <c r="I652" t="s">
-        <v>1694</v>
+        <v>1630</v>
       </c>
       <c r="J652" t="s">
-        <v>2378</v>
+        <v>2379</v>
       </c>
       <c r="K652" t="s">
-        <v>2483</v>
+        <v>2443</v>
       </c>
       <c r="L652" t="s">
-        <v>2526</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="653" spans="1:12">
       <c r="A653" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B653" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="C653" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="D653" t="s">
         <v>1593</v>
@@ -31140,30 +31140,30 @@
         <v>1602</v>
       </c>
       <c r="H653" t="s">
-        <v>1619</v>
+        <v>1622</v>
       </c>
       <c r="I653" t="s">
-        <v>1630</v>
+        <v>1743</v>
       </c>
       <c r="J653" t="s">
-        <v>2379</v>
+        <v>2380</v>
       </c>
       <c r="K653" t="s">
         <v>2443</v>
       </c>
       <c r="L653" t="s">
-        <v>2532</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="654" spans="1:12">
       <c r="A654" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B654" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C654" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="D654" t="s">
         <v>1593</v>
@@ -31172,36 +31172,33 @@
         <v>4</v>
       </c>
       <c r="F654" t="s">
-        <v>1598</v>
+        <v>1596</v>
       </c>
       <c r="G654" t="s">
-        <v>1602</v>
-      </c>
-      <c r="H654" t="s">
-        <v>1622</v>
+        <v>1601</v>
       </c>
       <c r="I654" t="s">
-        <v>1743</v>
+        <v>1723</v>
       </c>
       <c r="J654" t="s">
-        <v>2380</v>
+        <v>2381</v>
       </c>
       <c r="K654" t="s">
-        <v>2443</v>
+        <v>2522</v>
       </c>
       <c r="L654" t="s">
-        <v>2546</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B655" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="C655" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="D655" t="s">
         <v>1593</v>
@@ -31216,27 +31213,27 @@
         <v>1601</v>
       </c>
       <c r="I655" t="s">
-        <v>1723</v>
+        <v>1735</v>
       </c>
       <c r="J655" t="s">
-        <v>2381</v>
+        <v>2382</v>
       </c>
       <c r="K655" t="s">
-        <v>2522</v>
+        <v>2465</v>
       </c>
       <c r="L655" t="s">
-        <v>2548</v>
+        <v>2537</v>
       </c>
     </row>
     <row r="656" spans="1:12">
       <c r="A656" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B656" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="C656" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="D656" t="s">
         <v>1593</v>
@@ -31251,16 +31248,16 @@
         <v>1601</v>
       </c>
       <c r="I656" t="s">
-        <v>1735</v>
+        <v>1714</v>
       </c>
       <c r="J656" t="s">
-        <v>2382</v>
+        <v>2383</v>
       </c>
       <c r="K656" t="s">
-        <v>2465</v>
+        <v>2409</v>
       </c>
       <c r="L656" t="s">
-        <v>2537</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="657" spans="1:12">
@@ -31268,10 +31265,10 @@
         <v>23</v>
       </c>
       <c r="B657" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C657" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="D657" t="s">
         <v>1593</v>
@@ -31289,7 +31286,7 @@
         <v>1714</v>
       </c>
       <c r="J657" t="s">
-        <v>2383</v>
+        <v>2384</v>
       </c>
       <c r="K657" t="s">
         <v>2409</v>
@@ -31303,10 +31300,10 @@
         <v>23</v>
       </c>
       <c r="B658" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="C658" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="D658" t="s">
         <v>1593</v>
@@ -31324,7 +31321,7 @@
         <v>1714</v>
       </c>
       <c r="J658" t="s">
-        <v>2384</v>
+        <v>2385</v>
       </c>
       <c r="K658" t="s">
         <v>2409</v>
@@ -31338,10 +31335,10 @@
         <v>23</v>
       </c>
       <c r="B659" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="C659" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="D659" t="s">
         <v>1593</v>
@@ -31356,16 +31353,16 @@
         <v>1601</v>
       </c>
       <c r="I659" t="s">
-        <v>1714</v>
+        <v>1694</v>
       </c>
       <c r="J659" t="s">
-        <v>2385</v>
+        <v>2386</v>
       </c>
       <c r="K659" t="s">
-        <v>2409</v>
+        <v>2497</v>
       </c>
       <c r="L659" t="s">
-        <v>2582</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="660" spans="1:12">
@@ -31373,10 +31370,10 @@
         <v>23</v>
       </c>
       <c r="B660" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C660" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="D660" t="s">
         <v>1593</v>
@@ -31391,62 +31388,62 @@
         <v>1601</v>
       </c>
       <c r="I660" t="s">
-        <v>1694</v>
+        <v>1715</v>
       </c>
       <c r="J660" t="s">
-        <v>2386</v>
+        <v>2387</v>
       </c>
       <c r="K660" t="s">
-        <v>2497</v>
+        <v>2431</v>
       </c>
       <c r="L660" t="s">
-        <v>2526</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="661" spans="1:12">
       <c r="A661" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B661" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C661" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="D661" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="E661">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F661" t="s">
-        <v>1596</v>
+        <v>1600</v>
       </c>
       <c r="G661" t="s">
         <v>1601</v>
       </c>
       <c r="I661" t="s">
-        <v>1715</v>
+        <v>1744</v>
       </c>
       <c r="J661" t="s">
-        <v>2387</v>
+        <v>2388</v>
       </c>
       <c r="K661" t="s">
-        <v>2431</v>
+        <v>2406</v>
       </c>
       <c r="L661" t="s">
-        <v>2558</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="662" spans="1:12">
       <c r="A662" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="B662" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="C662" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="D662" t="s">
         <v>1594</v>
@@ -31455,33 +31452,33 @@
         <v>3</v>
       </c>
       <c r="F662" t="s">
-        <v>1600</v>
+        <v>1596</v>
       </c>
       <c r="G662" t="s">
         <v>1601</v>
       </c>
       <c r="I662" t="s">
-        <v>1744</v>
+        <v>1729</v>
       </c>
       <c r="J662" t="s">
-        <v>2388</v>
+        <v>2113</v>
       </c>
       <c r="K662" t="s">
-        <v>2406</v>
+        <v>2430</v>
       </c>
       <c r="L662" t="s">
-        <v>2567</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="663" spans="1:12">
       <c r="A663" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="B663" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C663" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="D663" t="s">
         <v>1594</v>
@@ -31496,16 +31493,16 @@
         <v>1601</v>
       </c>
       <c r="I663" t="s">
-        <v>1729</v>
+        <v>1735</v>
       </c>
       <c r="J663" t="s">
-        <v>2113</v>
+        <v>2389</v>
       </c>
       <c r="K663" t="s">
         <v>2430</v>
       </c>
       <c r="L663" t="s">
-        <v>2582</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="664" spans="1:12">
@@ -31513,10 +31510,10 @@
         <v>24</v>
       </c>
       <c r="B664" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="C664" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="D664" t="s">
         <v>1594</v>
@@ -31531,27 +31528,27 @@
         <v>1601</v>
       </c>
       <c r="I664" t="s">
-        <v>1735</v>
+        <v>1734</v>
       </c>
       <c r="J664" t="s">
-        <v>2389</v>
+        <v>2390</v>
       </c>
       <c r="K664" t="s">
         <v>2430</v>
       </c>
       <c r="L664" t="s">
-        <v>2557</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="665" spans="1:12">
       <c r="A665" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B665" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="C665" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
       <c r="D665" t="s">
         <v>1594</v>
@@ -31566,13 +31563,13 @@
         <v>1601</v>
       </c>
       <c r="I665" t="s">
-        <v>1734</v>
+        <v>1714</v>
       </c>
       <c r="J665" t="s">
-        <v>2390</v>
+        <v>2391</v>
       </c>
       <c r="K665" t="s">
-        <v>2430</v>
+        <v>2513</v>
       </c>
       <c r="L665" t="s">
         <v>2582</v>
@@ -31583,10 +31580,10 @@
         <v>23</v>
       </c>
       <c r="B666" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="C666" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="D666" t="s">
         <v>1594</v>
@@ -31601,16 +31598,16 @@
         <v>1601</v>
       </c>
       <c r="I666" t="s">
-        <v>1714</v>
+        <v>1731</v>
       </c>
       <c r="J666" t="s">
-        <v>2391</v>
+        <v>2392</v>
       </c>
       <c r="K666" t="s">
-        <v>2513</v>
+        <v>2420</v>
       </c>
       <c r="L666" t="s">
-        <v>2582</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="667" spans="1:12">
@@ -31618,10 +31615,10 @@
         <v>23</v>
       </c>
       <c r="B667" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="C667" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="D667" t="s">
         <v>1594</v>
@@ -31636,16 +31633,16 @@
         <v>1601</v>
       </c>
       <c r="I667" t="s">
-        <v>1731</v>
+        <v>1715</v>
       </c>
       <c r="J667" t="s">
-        <v>2392</v>
+        <v>2393</v>
       </c>
       <c r="K667" t="s">
-        <v>2420</v>
+        <v>2483</v>
       </c>
       <c r="L667" t="s">
-        <v>2527</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="668" spans="1:12">
@@ -31653,10 +31650,10 @@
         <v>23</v>
       </c>
       <c r="B668" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C668" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="D668" t="s">
         <v>1594</v>
@@ -31671,16 +31668,16 @@
         <v>1601</v>
       </c>
       <c r="I668" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="J668" t="s">
-        <v>2393</v>
+        <v>2394</v>
       </c>
       <c r="K668" t="s">
-        <v>2483</v>
+        <v>2457</v>
       </c>
       <c r="L668" t="s">
-        <v>2558</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="669" spans="1:12">
@@ -31688,16 +31685,16 @@
         <v>23</v>
       </c>
       <c r="B669" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C669" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="D669" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="E669">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F669" t="s">
         <v>1596</v>
@@ -31706,27 +31703,27 @@
         <v>1601</v>
       </c>
       <c r="I669" t="s">
-        <v>1714</v>
+        <v>1694</v>
       </c>
       <c r="J669" t="s">
-        <v>2394</v>
+        <v>2395</v>
       </c>
       <c r="K669" t="s">
-        <v>2457</v>
+        <v>2423</v>
       </c>
       <c r="L669" t="s">
-        <v>2582</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="670" spans="1:12">
       <c r="A670" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B670" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="C670" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
       <c r="D670" t="s">
         <v>1595</v>
@@ -31741,27 +31738,27 @@
         <v>1601</v>
       </c>
       <c r="I670" t="s">
-        <v>1694</v>
+        <v>1625</v>
       </c>
       <c r="J670" t="s">
-        <v>2395</v>
+        <v>2396</v>
       </c>
       <c r="K670" t="s">
-        <v>2423</v>
+        <v>2464</v>
       </c>
       <c r="L670" t="s">
-        <v>2526</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="671" spans="1:12">
       <c r="A671" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B671" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C671" t="s">
-        <v>1377</v>
+        <v>1378</v>
       </c>
       <c r="D671" t="s">
         <v>1595</v>
@@ -31776,13 +31773,13 @@
         <v>1601</v>
       </c>
       <c r="I671" t="s">
-        <v>1625</v>
+        <v>1739</v>
       </c>
       <c r="J671" t="s">
-        <v>2396</v>
+        <v>2397</v>
       </c>
       <c r="K671" t="s">
-        <v>2464</v>
+        <v>2523</v>
       </c>
       <c r="L671" t="s">
         <v>2582</v>
@@ -31793,10 +31790,10 @@
         <v>23</v>
       </c>
       <c r="B672" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C672" t="s">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="D672" t="s">
         <v>1595</v>
@@ -31814,10 +31811,10 @@
         <v>1739</v>
       </c>
       <c r="J672" t="s">
-        <v>2397</v>
+        <v>2398</v>
       </c>
       <c r="K672" t="s">
-        <v>2523</v>
+        <v>2524</v>
       </c>
       <c r="L672" t="s">
         <v>2582</v>
@@ -31828,10 +31825,10 @@
         <v>23</v>
       </c>
       <c r="B673" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="C673" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
       <c r="D673" t="s">
         <v>1595</v>
@@ -31843,33 +31840,33 @@
         <v>1596</v>
       </c>
       <c r="G673" t="s">
-        <v>1601</v>
+        <v>1602</v>
+      </c>
+      <c r="H673" t="s">
+        <v>1623</v>
       </c>
       <c r="I673" t="s">
-        <v>1739</v>
+        <v>1731</v>
       </c>
       <c r="J673" t="s">
-        <v>2398</v>
+        <v>2399</v>
       </c>
       <c r="K673" t="s">
-        <v>2524</v>
+        <v>2419</v>
       </c>
       <c r="L673" t="s">
-        <v>2582</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="674" spans="1:12">
       <c r="A674" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B674" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C674" t="s">
-        <v>1380</v>
-      </c>
-      <c r="D674" t="s">
-        <v>1595</v>
+        <v>1381</v>
       </c>
       <c r="E674">
         <v>0</v>
@@ -31878,22 +31875,19 @@
         <v>1596</v>
       </c>
       <c r="G674" t="s">
-        <v>1602</v>
-      </c>
-      <c r="H674" t="s">
-        <v>1623</v>
+        <v>1601</v>
       </c>
       <c r="I674" t="s">
-        <v>1731</v>
+        <v>1735</v>
       </c>
       <c r="J674" t="s">
-        <v>2399</v>
+        <v>2400</v>
       </c>
       <c r="K674" t="s">
-        <v>2419</v>
+        <v>2525</v>
       </c>
       <c r="L674" t="s">
-        <v>2527</v>
+        <v>2609</v>
       </c>
     </row>
     <row r="675" spans="1:12">
@@ -31901,10 +31895,10 @@
         <v>24</v>
       </c>
       <c r="B675" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C675" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="E675">
         <v>0</v>
@@ -31919,45 +31913,13 @@
         <v>1735</v>
       </c>
       <c r="J675" t="s">
-        <v>2400</v>
+        <v>2401</v>
       </c>
       <c r="K675" t="s">
         <v>2525</v>
       </c>
       <c r="L675" t="s">
         <v>2610</v>
-      </c>
-    </row>
-    <row r="676" spans="1:12">
-      <c r="A676" t="s">
-        <v>24</v>
-      </c>
-      <c r="B676" t="s">
-        <v>712</v>
-      </c>
-      <c r="C676" t="s">
-        <v>1382</v>
-      </c>
-      <c r="E676">
-        <v>0</v>
-      </c>
-      <c r="F676" t="s">
-        <v>1596</v>
-      </c>
-      <c r="G676" t="s">
-        <v>1601</v>
-      </c>
-      <c r="I676" t="s">
-        <v>1735</v>
-      </c>
-      <c r="J676" t="s">
-        <v>2401</v>
-      </c>
-      <c r="K676" t="s">
-        <v>2525</v>
-      </c>
-      <c r="L676" t="s">
-        <v>2611</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-01 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6714" uniqueCount="2598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6714" uniqueCount="2596">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -5128,12 +5128,12 @@
     <t>EDIWAN SOUSA DA SILVA,ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
   </si>
   <si>
+    <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
+  </si>
+  <si>
     <t>CHRISTIANA ROSA FERREIRA</t>
   </si>
   <si>
-    <t>VANESSA DOYNSILÊ LEAL DA SILVA</t>
-  </si>
-  <si>
     <t>RAQUEL SILVA FERNANDES LYRA</t>
   </si>
   <si>
@@ -7714,7 +7714,7 @@
     <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA CIVIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,URBANISMO</t>
@@ -7765,10 +7765,7 @@
     <t>MEDICINA LEGAL,SAÚDE</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
@@ -7780,6 +7777,9 @@
     <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
@@ -7789,25 +7789,19 @@
     <t>ASSISTÊNCIA SOCIAL,EDIFICAÇÕES</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
+    <t>ECONOMICIDADE OBRAS,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
     <t>SAÚDE,FARMÁCIA</t>
   </si>
   <si>
-    <t>SAÚDE,ORÇAMENTO</t>
-  </si>
-  <si>
     <t>URBANISMO,BIOLOGIA</t>
   </si>
   <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>ORÇAMENTO,PSICOLOGIA,URBANISMO,AVALIAÇÃO DE IMÓVEIS,MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL,SAÚDE,ECONOMIA,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL</t>
+    <t>ECONOMICIDADE CONTÁBIL,ORÇAMENTO,SAÚDE MENTAL,AVALIAÇÃO DE IMÓVEIS,SAÚDE,MOBILIDADE E TRANSPORTE,ECONOMIA,ASSISTÊNCIA SOCIAL,PSICOLOGIA,URBANISMO</t>
   </si>
 </sst>
 </file>
@@ -19913,7 +19907,7 @@
     </row>
     <row r="336" spans="1:12">
       <c r="A336" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B336" t="s">
         <v>378</v>
@@ -19934,7 +19928,7 @@
         <v>1587</v>
       </c>
       <c r="I336" t="s">
-        <v>1704</v>
+        <v>1613</v>
       </c>
       <c r="J336" t="s">
         <v>2070</v>
@@ -20074,7 +20068,7 @@
         <v>1587</v>
       </c>
       <c r="I340" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J340" t="s">
         <v>2074</v>
@@ -20599,7 +20593,7 @@
         <v>1587</v>
       </c>
       <c r="I355" t="s">
-        <v>1704</v>
+        <v>1705</v>
       </c>
       <c r="J355" t="s">
         <v>2089</v>
@@ -22603,7 +22597,7 @@
         <v>1587</v>
       </c>
       <c r="I412" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J412" t="s">
         <v>2146</v>
@@ -22813,7 +22807,7 @@
         <v>1587</v>
       </c>
       <c r="I418" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J418" t="s">
         <v>2152</v>
@@ -23338,7 +23332,7 @@
         <v>1587</v>
       </c>
       <c r="I433" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J433" t="s">
         <v>2166</v>
@@ -23408,7 +23402,7 @@
         <v>1587</v>
       </c>
       <c r="I435" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J435" t="s">
         <v>2168</v>
@@ -23417,7 +23411,7 @@
         <v>2399</v>
       </c>
       <c r="L435" t="s">
-        <v>2569</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="436" spans="1:12">
@@ -24041,7 +24035,7 @@
         <v>1587</v>
       </c>
       <c r="I453" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J453" t="s">
         <v>2186</v>
@@ -24225,7 +24219,7 @@
         <v>2433</v>
       </c>
       <c r="L458" t="s">
-        <v>2583</v>
+        <v>2579</v>
       </c>
     </row>
     <row r="459" spans="1:12">
@@ -24499,7 +24493,7 @@
         <v>1587</v>
       </c>
       <c r="I466" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J466" t="s">
         <v>2199</v>
@@ -24604,7 +24598,7 @@
         <v>1587</v>
       </c>
       <c r="I469" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J469" t="s">
         <v>2202</v>
@@ -24613,7 +24607,7 @@
         <v>2425</v>
       </c>
       <c r="L469" t="s">
-        <v>2569</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="470" spans="1:12">
@@ -24639,7 +24633,7 @@
         <v>1587</v>
       </c>
       <c r="I470" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J470" t="s">
         <v>2203</v>
@@ -25094,7 +25088,7 @@
         <v>1587</v>
       </c>
       <c r="I483" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J483" t="s">
         <v>2215</v>
@@ -25103,7 +25097,7 @@
         <v>2401</v>
       </c>
       <c r="L483" t="s">
-        <v>2569</v>
+        <v>2519</v>
       </c>
     </row>
     <row r="484" spans="1:12">
@@ -25797,7 +25791,7 @@
         <v>1587</v>
       </c>
       <c r="I503" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J503" t="s">
         <v>2235</v>
@@ -25806,7 +25800,7 @@
         <v>2412</v>
       </c>
       <c r="L503" t="s">
-        <v>2569</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="504" spans="1:12">
@@ -26996,7 +26990,7 @@
         <v>2489</v>
       </c>
       <c r="L537" t="s">
-        <v>2584</v>
+        <v>2583</v>
       </c>
     </row>
     <row r="538" spans="1:12">
@@ -27273,7 +27267,7 @@
         <v>1587</v>
       </c>
       <c r="I545" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J545" t="s">
         <v>2274</v>
@@ -27346,7 +27340,7 @@
         <v>1587</v>
       </c>
       <c r="I547" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J547" t="s">
         <v>2276</v>
@@ -27451,7 +27445,7 @@
         <v>1587</v>
       </c>
       <c r="I550" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J550" t="s">
         <v>2279</v>
@@ -27533,7 +27527,7 @@
         <v>2411</v>
       </c>
       <c r="L552" t="s">
-        <v>2585</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="553" spans="1:12">
@@ -27568,7 +27562,7 @@
         <v>2461</v>
       </c>
       <c r="L553" t="s">
-        <v>2586</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="554" spans="1:12">
@@ -28090,7 +28084,7 @@
         <v>1587</v>
       </c>
       <c r="I568" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J568" t="s">
         <v>2297</v>
@@ -28125,7 +28119,7 @@
         <v>1587</v>
       </c>
       <c r="I569" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J569" t="s">
         <v>2298</v>
@@ -28265,7 +28259,7 @@
         <v>1587</v>
       </c>
       <c r="I573" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J573" t="s">
         <v>2302</v>
@@ -28373,7 +28367,7 @@
         <v>1587</v>
       </c>
       <c r="I576" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J576" t="s">
         <v>2305</v>
@@ -28487,7 +28481,7 @@
         <v>2462</v>
       </c>
       <c r="L579" t="s">
-        <v>2587</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="580" spans="1:12">
@@ -28522,7 +28516,7 @@
         <v>2462</v>
       </c>
       <c r="L580" t="s">
-        <v>2587</v>
+        <v>2586</v>
       </c>
     </row>
     <row r="581" spans="1:12">
@@ -28557,7 +28551,7 @@
         <v>2406</v>
       </c>
       <c r="L581" t="s">
-        <v>2586</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="582" spans="1:12">
@@ -29575,7 +29569,7 @@
         <v>1587</v>
       </c>
       <c r="I610" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J610" t="s">
         <v>2335</v>
@@ -29791,7 +29785,7 @@
         <v>1587</v>
       </c>
       <c r="I616" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J616" t="s">
         <v>2341</v>
@@ -29931,7 +29925,7 @@
         <v>1587</v>
       </c>
       <c r="I620" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J620" t="s">
         <v>2345</v>
@@ -30080,7 +30074,7 @@
         <v>2503</v>
       </c>
       <c r="L624" t="s">
-        <v>2592</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="625" spans="1:12">
@@ -30115,7 +30109,7 @@
         <v>2435</v>
       </c>
       <c r="L625" t="s">
-        <v>2593</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="626" spans="1:12">
@@ -30217,7 +30211,7 @@
         <v>1606</v>
       </c>
       <c r="I628" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J628" t="s">
         <v>2352</v>
@@ -30325,7 +30319,7 @@
         <v>1587</v>
       </c>
       <c r="I631" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J631" t="s">
         <v>2355</v>
@@ -30407,7 +30401,7 @@
         <v>2467</v>
       </c>
       <c r="L633" t="s">
-        <v>2594</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -30433,7 +30427,7 @@
         <v>1587</v>
       </c>
       <c r="I634" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J634" t="s">
         <v>2358</v>
@@ -30442,7 +30436,7 @@
         <v>2431</v>
       </c>
       <c r="L634" t="s">
-        <v>2569</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="635" spans="1:12">
@@ -30754,7 +30748,7 @@
         <v>1587</v>
       </c>
       <c r="I643" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J643" t="s">
         <v>2367</v>
@@ -30789,7 +30783,7 @@
         <v>1587</v>
       </c>
       <c r="I644" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J644" t="s">
         <v>2368</v>
@@ -30824,7 +30818,7 @@
         <v>1587</v>
       </c>
       <c r="I645" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J645" t="s">
         <v>2369</v>
@@ -31069,7 +31063,7 @@
         <v>1587</v>
       </c>
       <c r="I652" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J652" t="s">
         <v>2375</v>
@@ -31174,7 +31168,7 @@
         <v>1587</v>
       </c>
       <c r="I655" t="s">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="J655" t="s">
         <v>2378</v>
@@ -31510,7 +31504,7 @@
         <v>2506</v>
       </c>
       <c r="L664" t="s">
-        <v>2595</v>
+        <v>2593</v>
       </c>
     </row>
     <row r="665" spans="1:12">
@@ -31612,7 +31606,7 @@
         <v>2514</v>
       </c>
       <c r="L667" t="s">
-        <v>2596</v>
+        <v>2594</v>
       </c>
     </row>
     <row r="668" spans="1:12">
@@ -31644,7 +31638,7 @@
         <v>2514</v>
       </c>
       <c r="L668" t="s">
-        <v>2597</v>
+        <v>2595</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-03 10:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7789,7 +7789,7 @@
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
@@ -7810,7 +7810,7 @@
     <t>ECONOMICIDADE CONTÁBIL,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
     <t>ECONOMICIDADE OBRAS,RECURSOS HÍDRICOS</t>
@@ -7825,6 +7825,9 @@
     <t>MEDICINA LEGAL,SAÚDE</t>
   </si>
   <si>
+    <t>RECURSOS HÍDRICOS,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
     <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
   </si>
   <si>
@@ -7834,19 +7837,19 @@
     <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
     <t>RECURSOS HÍDRICOS,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
-    <t>EDIFICAÇÕES,ASSISTÊNCIA SOCIAL</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
+    <t>ASSISTÊNCIA SOCIAL,EDIFICAÇÕES</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE OBRAS,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
     <t>FARMÁCIA,SAÚDE</t>
@@ -7855,10 +7858,7 @@
     <t>SAÚDE,ORÇAMENTO</t>
   </si>
   <si>
-    <t>URBANISMO,BIOLOGIA</t>
-  </si>
-  <si>
-    <t>ORÇAMENTO,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,ECONOMIA,URBANISMO,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,SAÚDE</t>
+    <t>SAÚDE MENTAL,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,ASSISTÊNCIA SOCIAL,ECONOMIA,SAÚDE,AVALIAÇÃO DE IMÓVEIS,MOBILIDADE E TRANSPORTE,URBANISMO,ORÇAMENTO</t>
   </si>
 </sst>
 </file>
@@ -24101,7 +24101,7 @@
         <v>2453</v>
       </c>
       <c r="L453" t="s">
-        <v>2599</v>
+        <v>2603</v>
       </c>
     </row>
     <row r="454" spans="1:12">
@@ -27409,7 +27409,7 @@
         <v>2430</v>
       </c>
       <c r="L547" t="s">
-        <v>2603</v>
+        <v>2604</v>
       </c>
     </row>
     <row r="548" spans="1:12">
@@ -27444,7 +27444,7 @@
         <v>2479</v>
       </c>
       <c r="L548" t="s">
-        <v>2604</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="549" spans="1:12">
@@ -28363,7 +28363,7 @@
         <v>2480</v>
       </c>
       <c r="L574" t="s">
-        <v>2605</v>
+        <v>2606</v>
       </c>
     </row>
     <row r="575" spans="1:12">
@@ -28398,7 +28398,7 @@
         <v>2480</v>
       </c>
       <c r="L575" t="s">
-        <v>2605</v>
+        <v>2606</v>
       </c>
     </row>
     <row r="576" spans="1:12">
@@ -28433,7 +28433,7 @@
         <v>2425</v>
       </c>
       <c r="L576" t="s">
-        <v>2604</v>
+        <v>2607</v>
       </c>
     </row>
     <row r="577" spans="1:12">
@@ -28468,7 +28468,7 @@
         <v>2521</v>
       </c>
       <c r="L577" t="s">
-        <v>2606</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="578" spans="1:12">
@@ -28859,7 +28859,7 @@
         <v>2420</v>
       </c>
       <c r="L588" t="s">
-        <v>2607</v>
+        <v>2609</v>
       </c>
     </row>
     <row r="589" spans="1:12">
@@ -29282,7 +29282,7 @@
         <v>2525</v>
       </c>
       <c r="L600" t="s">
-        <v>2608</v>
+        <v>2610</v>
       </c>
     </row>
     <row r="601" spans="1:12">
@@ -29425,7 +29425,7 @@
         <v>2448</v>
       </c>
       <c r="L604" t="s">
-        <v>2609</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="605" spans="1:12">
@@ -29956,7 +29956,7 @@
         <v>2520</v>
       </c>
       <c r="L619" t="s">
-        <v>2610</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29991,7 +29991,7 @@
         <v>2455</v>
       </c>
       <c r="L620" t="s">
-        <v>2611</v>
+        <v>2612</v>
       </c>
     </row>
     <row r="621" spans="1:12">
@@ -30283,7 +30283,7 @@
         <v>2484</v>
       </c>
       <c r="L628" t="s">
-        <v>2612</v>
+        <v>2613</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -31386,7 +31386,7 @@
         <v>2523</v>
       </c>
       <c r="L659" t="s">
-        <v>2613</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="660" spans="1:12">
@@ -31499,7 +31499,7 @@
     </row>
     <row r="663" spans="1:12">
       <c r="A663" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B663" t="s">
         <v>699</v>
@@ -31520,7 +31520,7 @@
         <v>1603</v>
       </c>
       <c r="I663" t="s">
-        <v>1630</v>
+        <v>1748</v>
       </c>
       <c r="J663" t="s">
         <v>2397</v>
@@ -31529,7 +31529,7 @@
         <v>2419</v>
       </c>
       <c r="L663" t="s">
-        <v>2588</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="664" spans="1:12">
@@ -31774,7 +31774,7 @@
         <v>2492</v>
       </c>
       <c r="L670" t="s">
-        <v>2588</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="671" spans="1:12">

</xml_diff>